<commit_message>
Add WBS Level 5 Family Policy CSV with detailed policy definitions and classifications
</commit_message>
<xml_diff>
--- a/data/raw/UNSCHEDULED EVENT CODE.xlsx
+++ b/data/raw/UNSCHEDULED EVENT CODE.xlsx
@@ -2535,10 +2535,10 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
     <TaxCatchAll xmlns="bf7de1ab-af5b-477c-916f-a25198a73d44" xsi:nil="true"/>
     <_Flow_SignoffStatus xmlns="eb1c4f4c-6ca0-42c7-8590-3fd2c794ca4e" xsi:nil="true"/>
-    <_dlc_DocId xmlns="bf7de1ab-af5b-477c-916f-a25198a73d44">E7CRSC4TRWZ4-297197074-23137518</_dlc_DocId>
+    <_dlc_DocId xmlns="bf7de1ab-af5b-477c-916f-a25198a73d44">E7CRSC4TRWZ4-297197074-23139185</_dlc_DocId>
     <_dlc_DocIdUrl xmlns="bf7de1ab-af5b-477c-916f-a25198a73d44">
-      <Url>https://starenergycoid.sharepoint.com/sites/STARDRIVE/_layouts/15/DocIdRedir.aspx?ID=E7CRSC4TRWZ4-297197074-23137518</Url>
-      <Description>E7CRSC4TRWZ4-297197074-23137518</Description>
+      <Url>https://starenergycoid.sharepoint.com/sites/STARDRIVE/_layouts/15/DocIdRedir.aspx?ID=E7CRSC4TRWZ4-297197074-23139185</Url>
+      <Description>E7CRSC4TRWZ4-297197074-23139185</Description>
     </_dlc_DocIdUrl>
   </documentManagement>
 </p:properties>

</xml_diff>